<commit_message>
Add concrete volume to all pipeline steps for walled structures
geometry.py: compute v_concrete for rectangular (outer box minus inner
void plus fillet area) and circular (annular ring) shapes; frustum has
none. run_tests.py: add assertions for B02 (152.673 m3) and B03
(116.113 m3), 32 checks all passing. main.py: add V_concrete column to
console table, frustum rows show n/a. exports.py: add column J Concrete
Volume (m3) with SUM formula in TOTAL row. charts.py: show V_c in 2D
blueprint labels and V_concrete annotation in 3D views. basin_template
rebuilt with 10-column layout (A-J).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/basin_template.xlsx
+++ b/basin_template.xlsx
@@ -26,16 +26,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -47,12 +45,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
+        <fgColor rgb="FF2E75B6"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,16 +64,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="FFAAAAAA"/>
       </left>
       <right style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="FFAAAAAA"/>
       </right>
       <top style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="FFAAAAAA"/>
       </top>
       <bottom style="thin">
-        <color rgb="00AAAAAA"/>
+        <color rgb="FFAAAAAA"/>
       </bottom>
     </border>
   </borders>
@@ -455,22 +453,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BASIN CALCULATION REPORT</t>
+          <t>Basin Geometry Calculation Summary</t>
         </is>
       </c>
     </row>
@@ -492,22 +493,37 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Raw Dimensions</t>
+          <t>Raw Input Dimensions</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Footprint</t>
+          <t>Length / Diameter (m)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Width (m)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Footprint Area (m2)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>Water Volume (m3)</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Total Excavation Volume (m3)</t>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Excavation Volume (m3)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Concrete Volume (m3)</t>
         </is>
       </c>
     </row>
@@ -532,15 +548,20 @@
           <t>L=20.0, 19.8, 20.2 W=10.0 h=5.0 slope=1.0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>30.00 × 20.00 m</t>
-        </is>
+      <c r="E3" t="n">
+        <v>30</v>
       </c>
       <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3">
+        <f>E3*F3</f>
+        <v/>
+      </c>
+      <c r="H3" t="n">
         <v>1464.18</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>1910.684</v>
       </c>
     </row>
@@ -565,15 +586,20 @@
           <t>L=20.0 W=10.0 h=5.0 slope=N0.0 S1.5 E1.0 W1.0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>30.00 × 17.50 m</t>
-        </is>
+      <c r="E4" t="n">
+        <v>30</v>
       </c>
       <c r="F4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G4">
+        <f>E4*F4</f>
+        <v/>
+      </c>
+      <c r="H4" t="n">
         <v>1354.075</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>1748.395</v>
       </c>
     </row>
@@ -598,16 +624,24 @@
           <t>L=25.0 W=12.0, 12.2 h=5.0 tw=0.4 R=0.5</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>25.80 × 12.90 m</t>
-        </is>
+      <c r="E5" t="n">
+        <v>25.8</v>
       </c>
       <c r="F5" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G5">
+        <f>E5*F5</f>
+        <v/>
+      </c>
+      <c r="H5" t="n">
         <v>1148.685</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>1664.1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>152.673</v>
       </c>
     </row>
     <row r="6">
@@ -631,16 +665,24 @@
           <t>D=15.0 h=6.0 tw=0.4</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Ø15.80 m</t>
-        </is>
+      <c r="E6" t="n">
+        <v>15.8</v>
       </c>
       <c r="F6" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="G6">
+        <f>PI()*(E6/2)^2</f>
+        <v/>
+      </c>
+      <c r="H6" t="n">
         <v>883.573</v>
       </c>
-      <c r="G6" t="n">
+      <c r="I6" t="n">
         <v>1176.401</v>
+      </c>
+      <c r="J6" t="n">
+        <v>116.113</v>
       </c>
     </row>
     <row r="7">
@@ -653,18 +695,27 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
-      <c r="F7">
-        <f>SUM(F3:F6)</f>
-        <v/>
-      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7">
         <f>SUM(G3:G6)</f>
         <v/>
       </c>
+      <c r="H7">
+        <f>SUM(H3:H6)</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>SUM(I3:I6)</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>SUM(J3:J6)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>